<commit_message>
grammar 1-3, double check
</commit_message>
<xml_diff>
--- a/GRAMMAR/1_21_07.xlsx
+++ b/GRAMMAR/1_21_07.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\N2_2025_12\GRAMMAR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB10749E-45F2-4E73-AD9B-8A6FD333EA14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E54AB528-0C3A-4356-8CC0-0539ED3F006A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10560" yWindow="915" windowWidth="27840" windowHeight="20040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="1560" windowWidth="27840" windowHeight="20040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -278,9 +278,6 @@
   </si>
   <si>
     <t>をとわず</t>
-  </si>
-  <si>
-    <t>にあたって</t>
   </si>
   <si>
     <t>在……之际(重要时刻)</t>
@@ -498,12 +495,36 @@
     <t>(1)发现(2)如果</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">动词原形 + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>にあたって</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -541,6 +562,13 @@
       <family val="2"/>
       <charset val="128"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1081,13 +1109,13 @@
         <v>2</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.15">
@@ -1373,10 +1401,10 @@
         <v>0</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="D38" s="2"/>
     </row>
@@ -1385,13 +1413,13 @@
         <v>0</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="D39" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.15">
@@ -1399,13 +1427,13 @@
         <v>0</v>
       </c>
       <c r="B40" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="D40" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.15">
@@ -1413,10 +1441,10 @@
         <v>0</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="D41" s="2"/>
     </row>
@@ -1425,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="D42" s="2"/>
     </row>
@@ -1437,10 +1465,10 @@
         <v>0</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="D43" s="2"/>
     </row>
@@ -1449,13 +1477,13 @@
         <v>0</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="D44" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.15">
@@ -1463,10 +1491,10 @@
         <v>0</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="D45" s="2"/>
     </row>
@@ -1475,10 +1503,10 @@
         <v>0</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>106</v>
       </c>
       <c r="D46" s="2"/>
     </row>
@@ -1487,10 +1515,10 @@
         <v>0</v>
       </c>
       <c r="B47" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="D47" s="2"/>
     </row>
@@ -1499,10 +1527,10 @@
         <v>0</v>
       </c>
       <c r="B48" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>14</v>
@@ -1513,10 +1541,10 @@
         <v>0</v>
       </c>
       <c r="B49" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="D49" s="2"/>
     </row>
@@ -1525,10 +1553,10 @@
         <v>0</v>
       </c>
       <c r="B50" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="D50" s="2"/>
     </row>
@@ -1537,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="B51" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C51" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="D51" s="2"/>
     </row>
@@ -1549,10 +1577,10 @@
         <v>0</v>
       </c>
       <c r="B52" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="D52" s="2"/>
     </row>
@@ -1564,10 +1592,10 @@
         <v>41</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.15">
@@ -1575,10 +1603,10 @@
         <v>2</v>
       </c>
       <c r="B54" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="D54" s="2"/>
     </row>
@@ -1587,10 +1615,10 @@
         <v>2</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D55" s="2"/>
     </row>
@@ -1599,10 +1627,10 @@
         <v>2</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D56" s="2"/>
     </row>
@@ -1611,10 +1639,10 @@
         <v>2</v>
       </c>
       <c r="B57" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>128</v>
       </c>
       <c r="D57" s="2"/>
     </row>

</xml_diff>